<commit_message>
February Run Some code changes were made. Also made decision to gitignore the temp folder
</commit_message>
<xml_diff>
--- a/code/Monthly processing worksheet.xlsx
+++ b/code/Monthly processing worksheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ExecutiveSearchYaml\code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{39F5D6DA-8584-4675-A7D0-D2C69EF5FD11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FBD3447-76F8-4E33-AAF9-040871C1ACBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20330" yWindow="1250" windowWidth="15340" windowHeight="17860" xr2:uid="{DE42545E-C2A1-4C29-B894-0BEAE1CA5317}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="66">
   <si>
     <t>MONTHLY EXECUTIVE DATA COLLECTION - COMPLETE WORKFLOW</t>
   </si>
@@ -291,6 +291,9 @@
   </si>
   <si>
     <t>Manual spot-checks, compare with previous month</t>
+  </si>
+  <si>
+    <t>Recovery process</t>
   </si>
 </sst>
 </file>
@@ -719,7 +722,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{040A7AA3-A2C3-4733-A23A-F1BFE48DEF92}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="16.6328125" customWidth="1"/>
@@ -1008,6 +1011,11 @@
       </c>
       <c r="G21" s="4" t="s">
         <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="B22" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>